<commit_message>
Statusul fluxurilor scapa de istoricul de livrare
Coloana Status purta '(Etapa 1/2/3/4)' -- ordinea in care au fost scrise, nu
starea fluxului. Iese din foaia de lucru si se pastreaza integral in Istoric, pe
o coloana proprie. Marcajele CORECTAT / CLARIFICAT raman: acelea spun ceva despre
continut, nu despre cronologie.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XUbema9LnEV5DwY3Zjnxhc
</commit_message>
<xml_diff>
--- a/dist/Plan_de_conturi_ROL_Analitice_Fluxuri_SAGA.xlsx
+++ b/dist/Plan_de_conturi_ROL_Analitice_Fluxuri_SAGA.xlsx
@@ -1905,7 +1905,7 @@
     <row r="5">
       <c r="A5" s="62" t="inlineStr">
         <is>
-          <t>Numerotarea veche era secvențială, în ordinea livrărilor. Cea nouă codifică clasa contului principal, deci un flux adăugat peste un an primește următorul număr liber din clasa lui și stă fizic la locul lui. Tabelul rămâne aici permanent, ca referințele vechi să se poată rezolva.</t>
+          <t>Numerotarea veche era secvențială, în ordinea livrărilor. Cea nouă codifică clasa contului principal, deci un flux adăugat peste un an primește următorul număr liber din clasa lui și stă fizic la locul lui. Tabelul rămâne aici permanent, ca referințele vechi să se poată rezolva. Ultima coloană păstrează statusul dinainte de curățare: „(Etapa N)” era istoric de livrare, nu stare a fluxului, deci a ieșit din foaia de lucru.</t>
         </is>
       </c>
     </row>
@@ -1930,6 +1930,11 @@
           <t>Denumire</t>
         </is>
       </c>
+      <c r="E6" s="66" t="inlineStr">
+        <is>
+          <t>Status original (înainte de curățare)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="67" t="inlineStr">
@@ -1950,6 +1955,11 @@
           <t>Constituire / majorare capital social</t>
         </is>
       </c>
+      <c r="E7" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="67" t="inlineStr">
@@ -1970,6 +1980,11 @@
           <t>Rezerve din reevaluare: 105 → 1175</t>
         </is>
       </c>
+      <c r="E8" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="67" t="inlineStr">
@@ -1990,6 +2005,11 @@
           <t>Repartizarea rezultatului: 121 → 129/1061 → 1171</t>
         </is>
       </c>
+      <c r="E9" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="67" t="inlineStr">
@@ -2010,6 +2030,11 @@
           <t>Închiderea exercițiului (121/129/117 + 691/697/4417)</t>
         </is>
       </c>
+      <c r="E10" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 1)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="67" t="inlineStr">
@@ -2030,6 +2055,11 @@
           <t>Corecția erorilor din exerciții anterioare (1174)</t>
         </is>
       </c>
+      <c r="E11" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="67" t="inlineStr">
@@ -2050,6 +2080,11 @@
           <t>Provizioane pentru litigii (151x)</t>
         </is>
       </c>
+      <c r="E12" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="67" t="inlineStr">
@@ -2070,6 +2105,11 @@
           <t>Credit bancar în valută (162x)</t>
         </is>
       </c>
+      <c r="E13" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="67" t="inlineStr">
@@ -2090,6 +2130,11 @@
           <t>Leasing financiar autoturism cu deductibilitate 50%</t>
         </is>
       </c>
+      <c r="E14" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="67" t="inlineStr">
@@ -2110,6 +2155,11 @@
           <t>Imobilizări necorporale (20x)</t>
         </is>
       </c>
+      <c r="E15" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="67" t="inlineStr">
@@ -2130,6 +2180,11 @@
           <t>Terenuri și amenajări de terenuri (211)</t>
         </is>
       </c>
+      <c r="E16" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="67" t="inlineStr">
@@ -2150,6 +2205,11 @@
           <t>Construcții (212)</t>
         </is>
       </c>
+      <c r="E17" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="67" t="inlineStr">
@@ -2170,6 +2230,11 @@
           <t>Achiziție mijloc fix intern + amortizare liniară</t>
         </is>
       </c>
+      <c r="E18" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 3)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="67" t="inlineStr">
@@ -2190,6 +2255,11 @@
           <t>Instalații tehnice și mijloace de transport (213)</t>
         </is>
       </c>
+      <c r="E19" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="67" t="inlineStr">
@@ -2210,6 +2280,11 @@
           <t>Investiții imobiliare (215) și defalcarea teren / construcție</t>
         </is>
       </c>
+      <c r="E20" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="67" t="inlineStr">
@@ -2230,6 +2305,11 @@
           <t>Imobilizări facturate dar nesosite (223 / 224)</t>
         </is>
       </c>
+      <c r="E21" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="67" t="inlineStr">
@@ -2250,6 +2330,11 @@
           <t>Imobilizări în curs de execuție (231)</t>
         </is>
       </c>
+      <c r="E22" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="67" t="inlineStr">
@@ -2270,6 +2355,11 @@
           <t>Producție de imobilizări în regie proprie (722)</t>
         </is>
       </c>
+      <c r="E23" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 2) | CORECTAT 14.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="67" t="inlineStr">
@@ -2290,6 +2380,11 @@
           <t>Subvenție 475 eliberată pe măsura amortizării</t>
         </is>
       </c>
+      <c r="E24" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 1)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="67" t="inlineStr">
@@ -2310,6 +2405,11 @@
           <t>Vânzarea unui mijloc fix și testul valorii rămase</t>
         </is>
       </c>
+      <c r="E25" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="67" t="inlineStr">
@@ -2330,6 +2430,11 @@
           <t>Casarea unui mijloc fix și piesele recuperate</t>
         </is>
       </c>
+      <c r="E26" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="67" t="inlineStr">
@@ -2350,6 +2455,11 @@
           <t>Imobilizări financiare (26x)</t>
         </is>
       </c>
+      <c r="E27" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="67" t="inlineStr">
@@ -2370,6 +2480,11 @@
           <t>Controlul lunar analitic ↔ sintetic la imobilizări</t>
         </is>
       </c>
+      <c r="E28" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 4)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="67" t="inlineStr">
@@ -2390,6 +2505,11 @@
           <t>Aprovizionare internă (fără tranzit)</t>
         </is>
       </c>
+      <c r="E29" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="67" t="inlineStr">
@@ -2410,6 +2530,11 @@
           <t>Aprovizionare prin 32x (tranzit)</t>
         </is>
       </c>
+      <c r="E30" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 1)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="67" t="inlineStr">
@@ -2430,6 +2555,11 @@
           <t>Aprovizionare intracomunitară cu taxare inversă</t>
         </is>
       </c>
+      <c r="E31" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="67" t="inlineStr">
@@ -2450,6 +2580,11 @@
           <t>Intersecție 32x ↔ 408 (marfă parțială)</t>
         </is>
       </c>
+      <c r="E32" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="67" t="inlineStr">
@@ -2470,6 +2605,11 @@
           <t>Obiecte de inventar cu 8035 cap-coadă</t>
         </is>
       </c>
+      <c r="E33" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="67" t="inlineStr">
@@ -2490,6 +2630,11 @@
           <t>Diferențe de preț 308 / 348</t>
         </is>
       </c>
+      <c r="E34" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="67" t="inlineStr">
@@ -2510,6 +2655,11 @@
           <t>Ajustare pentru deprecierea stocurilor</t>
         </is>
       </c>
+      <c r="E35" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="67" t="inlineStr">
@@ -2530,6 +2680,11 @@
           <t>Piese de schimb 3024 → 371</t>
         </is>
       </c>
+      <c r="E36" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="67" t="inlineStr">
@@ -2550,6 +2705,11 @@
           <t>Stocuri aflate la terți</t>
         </is>
       </c>
+      <c r="E37" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="67" t="inlineStr">
@@ -2570,6 +2730,11 @@
           <t>Ambalaje + taxa AFM</t>
         </is>
       </c>
+      <c r="E38" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="67" t="inlineStr">
@@ -2590,6 +2755,11 @@
           <t>Producție termopan multi-stadiu (331 → 711 → 345)</t>
         </is>
       </c>
+      <c r="E39" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 1) | CORECTAT 14.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="67" t="inlineStr">
@@ -2610,6 +2780,11 @@
           <t>Servicii în curs 332 / 712</t>
         </is>
       </c>
+      <c r="E40" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 2) | CORECTAT 14.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="67" t="inlineStr">
@@ -2630,6 +2805,11 @@
           <t>Deșeuri 346</t>
         </is>
       </c>
+      <c r="E41" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 2) | CORECTAT 14.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="67" t="inlineStr">
@@ -2650,6 +2830,11 @@
           <t>Sold 331 la 31.12 → inventar → reluare ianuarie</t>
         </is>
       </c>
+      <c r="E42" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="67" t="inlineStr">
@@ -2670,6 +2855,11 @@
           <t>Vânzare en-gros</t>
         </is>
       </c>
+      <c r="E43" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="67" t="inlineStr">
@@ -2690,6 +2880,11 @@
           <t>Gestiune amănunt completă</t>
         </is>
       </c>
+      <c r="E44" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="67" t="inlineStr">
@@ -2710,6 +2905,11 @@
           <t>Vânzare parțială amănunt</t>
         </is>
       </c>
+      <c r="E45" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="67" t="inlineStr">
@@ -2730,6 +2930,11 @@
           <t>Retur din gestiune amănunt</t>
         </is>
       </c>
+      <c r="E46" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="67" t="inlineStr">
@@ -2750,6 +2955,11 @@
           <t>Import prin comisionar (446.VAMA)</t>
         </is>
       </c>
+      <c r="E47" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 1) | CORECTAT 14.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="67" t="inlineStr">
@@ -2770,6 +2980,11 @@
           <t>Import cu plată directă în vamă</t>
         </is>
       </c>
+      <c r="E48" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 3) | CORECTAT 14.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="67" t="inlineStr">
@@ -2790,6 +3005,11 @@
           <t>TVA la încasare (4428.INC)</t>
         </is>
       </c>
+      <c r="E49" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 1)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="67" t="inlineStr">
@@ -2810,6 +3030,11 @@
           <t>Taxare inversă internă</t>
         </is>
       </c>
+      <c r="E50" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 3)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="67" t="inlineStr">
@@ -2830,6 +3055,11 @@
           <t>Livrare intracomunitară scutită</t>
         </is>
       </c>
+      <c r="E51" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 3)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="67" t="inlineStr">
@@ -2850,6 +3080,11 @@
           <t>Export</t>
         </is>
       </c>
+      <c r="E52" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 3)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="67" t="inlineStr">
@@ -2870,6 +3105,11 @@
           <t>Închiderea lunară de TVA</t>
         </is>
       </c>
+      <c r="E53" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="67" t="inlineStr">
@@ -2890,6 +3130,11 @@
           <t>Înregistrări fără document (50% auto, lipsă la inventar)</t>
         </is>
       </c>
+      <c r="E54" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 3) | CORECTAT 14.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="67" t="inlineStr">
@@ -2910,6 +3155,11 @@
           <t>Corecție după D300 depusă</t>
         </is>
       </c>
+      <c r="E55" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="67" t="inlineStr">
@@ -2930,6 +3180,11 @@
           <t>408 / 418 (facturi nesosite / de întocmit)</t>
         </is>
       </c>
+      <c r="E56" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 1)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="67" t="inlineStr">
@@ -2950,6 +3205,11 @@
           <t>Reduceri comerciale 609 / 709</t>
         </is>
       </c>
+      <c r="E57" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 3) | CORECTAT 14.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="67" t="inlineStr">
@@ -2970,6 +3230,11 @@
           <t>Avansuri clienți / furnizori (419 / 409)</t>
         </is>
       </c>
+      <c r="E58" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 3) | CLARIFICAT 14.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="67" t="inlineStr">
@@ -2990,6 +3255,11 @@
           <t>Sumă neidentificată din extras → 473</t>
         </is>
       </c>
+      <c r="E59" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 1)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="67" t="inlineStr">
@@ -3010,6 +3280,11 @@
           <t>Avansuri 471 / 472 (regularizare temporală)</t>
         </is>
       </c>
+      <c r="E60" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 3)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="67" t="inlineStr">
@@ -3030,6 +3305,11 @@
           <t>Salarii</t>
         </is>
       </c>
+      <c r="E61" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 3)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="67" t="inlineStr">
@@ -3050,6 +3330,11 @@
           <t>Decontări 481 / 482 (unitate ↔ subunități)</t>
         </is>
       </c>
+      <c r="E62" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 3)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="67" t="inlineStr">
@@ -3070,6 +3355,11 @@
           <t>Viramente interne 581</t>
         </is>
       </c>
+      <c r="E63" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 1)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="67" t="inlineStr">
@@ -3090,6 +3380,11 @@
           <t>Avansuri de trezorerie (542)</t>
         </is>
       </c>
+      <c r="E64" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 3)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="67" t="inlineStr">
@@ -3110,6 +3405,11 @@
           <t>Angajamente extrabilanțiere</t>
         </is>
       </c>
+      <c r="E65" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat (Etapa 3)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="67" t="inlineStr">
@@ -3128,6 +3428,11 @@
       <c r="D66" s="67" t="inlineStr">
         <is>
           <t>Inventariere 8035 (scriptic vs. faptic)</t>
+        </is>
+      </c>
+      <c r="E66" s="67" t="inlineStr">
+        <is>
+          <t>Detaliat</t>
         </is>
       </c>
     </row>
@@ -22318,7 +22623,7 @@
       </c>
       <c r="G11" s="69" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H11" s="69" t="inlineStr">
@@ -22358,7 +22663,7 @@
       </c>
       <c r="G12" s="69" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H12" s="69" t="inlineStr">
@@ -22398,7 +22703,7 @@
       </c>
       <c r="G13" s="70" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H13" s="70" t="inlineStr">
@@ -22438,7 +22743,7 @@
       </c>
       <c r="G14" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 1)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H14" s="29" t="inlineStr">
@@ -22478,7 +22783,7 @@
       </c>
       <c r="G15" s="70" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H15" s="70" t="inlineStr">
@@ -22518,7 +22823,7 @@
       </c>
       <c r="G16" s="69" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H16" s="69" t="inlineStr">
@@ -22558,7 +22863,7 @@
       </c>
       <c r="G17" s="70" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H17" s="70" t="inlineStr">
@@ -22598,7 +22903,7 @@
       </c>
       <c r="G18" s="70" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H18" s="70" t="inlineStr">
@@ -22645,7 +22950,7 @@
       </c>
       <c r="G20" s="70" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H20" s="70" t="inlineStr">
@@ -22685,7 +22990,7 @@
       </c>
       <c r="G21" s="69" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H21" s="69" t="inlineStr">
@@ -22725,7 +23030,7 @@
       </c>
       <c r="G22" s="70" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H22" s="70" t="inlineStr">
@@ -22765,7 +23070,7 @@
       </c>
       <c r="G23" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 3)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H23" s="23" t="inlineStr">
@@ -22805,7 +23110,7 @@
       </c>
       <c r="G24" s="69" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H24" s="69" t="inlineStr">
@@ -22845,7 +23150,7 @@
       </c>
       <c r="G25" s="69" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H25" s="69" t="inlineStr">
@@ -22885,7 +23190,7 @@
       </c>
       <c r="G26" s="69" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H26" s="69" t="inlineStr">
@@ -22925,7 +23230,7 @@
       </c>
       <c r="G27" s="70" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H27" s="70" t="inlineStr">
@@ -22965,7 +23270,7 @@
       </c>
       <c r="G28" s="23" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 2) | CORECTAT 14.08.2026</t>
+          <t>Detaliat | CORECTAT 14.08.2026</t>
         </is>
       </c>
       <c r="H28" s="29" t="inlineStr">
@@ -23005,7 +23310,7 @@
       </c>
       <c r="G29" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 1)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H29" s="29" t="inlineStr">
@@ -23045,7 +23350,7 @@
       </c>
       <c r="G30" s="70" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H30" s="70" t="inlineStr">
@@ -23085,7 +23390,7 @@
       </c>
       <c r="G31" s="69" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H31" s="69" t="inlineStr">
@@ -23125,7 +23430,7 @@
       </c>
       <c r="G32" s="69" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H32" s="69" t="inlineStr">
@@ -23165,7 +23470,7 @@
       </c>
       <c r="G33" s="70" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 4)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H33" s="70" t="inlineStr">
@@ -23212,7 +23517,7 @@
       </c>
       <c r="G35" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 2)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H35" s="28" t="inlineStr">
@@ -23252,7 +23557,7 @@
       </c>
       <c r="G36" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 1)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H36" s="29" t="inlineStr">
@@ -23292,7 +23597,7 @@
       </c>
       <c r="G37" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 2)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H37" s="28" t="inlineStr">
@@ -23612,7 +23917,7 @@
       </c>
       <c r="G45" s="23" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 1) | CORECTAT 14.08.2026</t>
+          <t>Detaliat | CORECTAT 14.08.2026</t>
         </is>
       </c>
       <c r="H45" s="29" t="inlineStr">
@@ -23652,7 +23957,7 @@
       </c>
       <c r="G46" s="23" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 2) | CORECTAT 14.08.2026</t>
+          <t>Detaliat | CORECTAT 14.08.2026</t>
         </is>
       </c>
       <c r="H46" s="23" t="inlineStr">
@@ -23697,7 +24002,7 @@
       </c>
       <c r="G47" s="23" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 2) | CORECTAT 14.08.2026</t>
+          <t>Detaliat | CORECTAT 14.08.2026</t>
         </is>
       </c>
       <c r="H47" s="28" t="inlineStr">
@@ -23937,7 +24242,7 @@
       </c>
       <c r="G53" s="23" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 1) | CORECTAT 14.08.2026</t>
+          <t>Detaliat | CORECTAT 14.08.2026</t>
         </is>
       </c>
       <c r="H53" s="29" t="inlineStr">
@@ -23977,7 +24282,7 @@
       </c>
       <c r="G54" s="23" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 3) | CORECTAT 14.08.2026</t>
+          <t>Detaliat | CORECTAT 14.08.2026</t>
         </is>
       </c>
       <c r="H54" s="30" t="inlineStr">
@@ -24024,7 +24329,7 @@
       </c>
       <c r="G56" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 1)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H56" s="29" t="inlineStr">
@@ -24064,7 +24369,7 @@
       </c>
       <c r="G57" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 3)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H57" s="30" t="inlineStr">
@@ -24104,7 +24409,7 @@
       </c>
       <c r="G58" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 3)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H58" s="30" t="inlineStr">
@@ -24144,7 +24449,7 @@
       </c>
       <c r="G59" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 3)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H59" s="30" t="inlineStr">
@@ -24224,7 +24529,7 @@
       </c>
       <c r="G61" s="23" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 3) | CORECTAT 14.08.2026</t>
+          <t>Detaliat | CORECTAT 14.08.2026</t>
         </is>
       </c>
       <c r="H61" s="30" t="inlineStr">
@@ -24304,7 +24609,7 @@
       </c>
       <c r="G63" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 1)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H63" s="29" t="inlineStr">
@@ -24344,7 +24649,7 @@
       </c>
       <c r="G64" s="23" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 3) | CORECTAT 14.08.2026</t>
+          <t>Detaliat | CORECTAT 14.08.2026</t>
         </is>
       </c>
       <c r="H64" s="30" t="inlineStr">
@@ -24384,7 +24689,7 @@
       </c>
       <c r="G65" s="23" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 3) | CLARIFICAT 14.08.2026</t>
+          <t>Detaliat | CLARIFICAT 14.08.2026</t>
         </is>
       </c>
       <c r="H65" s="30" t="inlineStr">
@@ -24424,7 +24729,7 @@
       </c>
       <c r="G66" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 1)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H66" s="29" t="inlineStr">
@@ -24464,7 +24769,7 @@
       </c>
       <c r="G67" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 3)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H67" s="23" t="inlineStr">
@@ -24504,7 +24809,7 @@
       </c>
       <c r="G68" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 3)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H68" s="23" t="inlineStr">
@@ -24544,7 +24849,7 @@
       </c>
       <c r="G69" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 3)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H69" s="23" t="inlineStr">
@@ -24591,7 +24896,7 @@
       </c>
       <c r="G71" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 1)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H71" s="29" t="inlineStr">
@@ -24631,7 +24936,7 @@
       </c>
       <c r="G72" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 3)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H72" s="23" t="inlineStr">
@@ -24678,7 +24983,7 @@
       </c>
       <c r="G74" s="29" t="inlineStr">
         <is>
-          <t>Detaliat (Etapa 3)</t>
+          <t>Detaliat</t>
         </is>
       </c>
       <c r="H74" s="23" t="inlineStr">

</xml_diff>